<commit_message>
pnr status check - manual testcases added
</commit_message>
<xml_diff>
--- a/ApabritaSarkar_RedBus/ManualTesting/ApabritaSarkar_Epic1.xlsx
+++ b/ApabritaSarkar_RedBus/ManualTesting/ApabritaSarkar_Epic1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\OneDrive\Desktop\cg_training\Sprint\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\OneDrive\Desktop\cg_training\Sprint\DAY5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC45A8C7-1C42-4B8A-8D1F-84A490D1BF4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2B01E10-5CF1-4F2C-9435-5371DF99EADC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="User Stories" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="Test Cases" sheetId="3" r:id="rId3"/>
     <sheet name="Defect Report" sheetId="4" r:id="rId4"/>
     <sheet name="RTM" sheetId="5" r:id="rId5"/>
+    <sheet name="Summary" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="304">
   <si>
     <t>Issue Type</t>
   </si>
@@ -726,9 +727,6 @@
     <t>DF_02</t>
   </si>
   <si>
-    <t>DF_03</t>
-  </si>
-  <si>
     <t>TC_09</t>
   </si>
   <si>
@@ -815,13 +813,203 @@
   </si>
   <si>
     <t>Todo</t>
+  </si>
+  <si>
+    <t>TEST EXECUTION SUMMARY</t>
+  </si>
+  <si>
+    <t>Project Name</t>
+  </si>
+  <si>
+    <t>Module Name</t>
+  </si>
+  <si>
+    <t>Total Cases</t>
+  </si>
+  <si>
+    <t>Total Passed</t>
+  </si>
+  <si>
+    <t>Total Failed</t>
+  </si>
+  <si>
+    <t>Total Executed</t>
+  </si>
+  <si>
+    <t>Pass Percentage</t>
+  </si>
+  <si>
+    <t>Fail Percentage</t>
+  </si>
+  <si>
+    <t>Live Train Status</t>
+  </si>
+  <si>
+    <t>Top 10 Trains &amp; Seat Availability</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
+  </si>
+  <si>
+    <t>Date Selection &amp; Calendar</t>
+  </si>
+  <si>
+    <t>S-01.4</t>
+  </si>
+  <si>
+    <t>User checks PNR status to view booking details</t>
+  </si>
+  <si>
+    <t>SS-01.4.1</t>
+  </si>
+  <si>
+    <t>SS-01.4.2</t>
+  </si>
+  <si>
+    <t>Enter valid 10-digit PNR and view status</t>
+  </si>
+  <si>
+    <t>Show error for invalid PNR</t>
+  </si>
+  <si>
+    <t>SS-01.4.3</t>
+  </si>
+  <si>
+    <t>SS-01.4.4</t>
+  </si>
+  <si>
+    <t>Restrict input to exactly 10 digits</t>
+  </si>
+  <si>
+    <t>Disable button for incomplete PNR</t>
+  </si>
+  <si>
+    <t>TS_07</t>
+  </si>
+  <si>
+    <t>REQ_SS-01.4</t>
+  </si>
+  <si>
+    <t>PNR Status Check</t>
+  </si>
+  <si>
+    <t>1. Valid 10-digit PNR
+2. Invalid 10-digit PNR (neg)
+3. Less than 10 digits (neg)
+4. More than 10 digits restricted</t>
+  </si>
+  <si>
+    <t>TC_22</t>
+  </si>
+  <si>
+    <t>TC_23</t>
+  </si>
+  <si>
+    <t>TC_24</t>
+  </si>
+  <si>
+    <t>TC_25</t>
+  </si>
+  <si>
+    <t>App open, PNR section visible</t>
+  </si>
+  <si>
+    <t>Valid 10-digit PNR</t>
+  </si>
+  <si>
+    <t>1. Open PNR Check
+2. Enter PNR → 6700914458
+3. Click "Check Status"</t>
+  </si>
+  <si>
+    <t>PNR status page opens with booking details</t>
+  </si>
+  <si>
+    <t>PNR: 6700914458</t>
+  </si>
+  <si>
+    <t>PNR status displayed</t>
+  </si>
+  <si>
+    <t>REQ_SS-01.4.1</t>
+  </si>
+  <si>
+    <t>Invalid 10-digit PNR</t>
+  </si>
+  <si>
+    <t>1. Open PNR Check
+2. Enter PNR → 3476986918
+3. Click "Check Status"</t>
+  </si>
+  <si>
+    <t>PNR: 3476986918</t>
+  </si>
+  <si>
+    <t>Error message displayed: "Incorrect PNR Number"</t>
+  </si>
+  <si>
+    <t>Error message shown</t>
+  </si>
+  <si>
+    <t>Less than 10 digits</t>
+  </si>
+  <si>
+    <t>Check Status button disabled</t>
+  </si>
+  <si>
+    <t>1. Open PNR Check
+2. Enter PNR → 1234
+3. Try to click "Check Status"</t>
+  </si>
+  <si>
+    <t>incomplete PNR: 1234</t>
+  </si>
+  <si>
+    <t>Button disabled</t>
+  </si>
+  <si>
+    <t>More than 10 digits</t>
+  </si>
+  <si>
+    <t>Try entering 1234567890123</t>
+  </si>
+  <si>
+    <t>1. Open PNR Check
+2. Try entering 1234567890123</t>
+  </si>
+  <si>
+    <t>Input restricted to 10 digits</t>
+  </si>
+  <si>
+    <t>Only 10 digits accepted</t>
+  </si>
+  <si>
+    <t>REQ_SS-01.4.2</t>
+  </si>
+  <si>
+    <t>REQ_SS-01.4.3</t>
+  </si>
+  <si>
+    <t>REQ_SS-01.4.4</t>
+  </si>
+  <si>
+    <t>BR_07</t>
+  </si>
+  <si>
+    <t>TR_07</t>
+  </si>
+  <si>
+    <t>`1</t>
+  </si>
+  <si>
+    <t>Completion Percentage</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -903,6 +1091,20 @@
       <family val="2"/>
     </font>
     <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF375623"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="10"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -913,8 +1115,15 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="27">
+  <fills count="32">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1019,8 +1228,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF1F497D"/>
+        <bgColor rgb="FF1F497D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
         <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEEF3F8"/>
+        <bgColor rgb="FFEEF3F8"/>
       </patternFill>
     </fill>
     <fill>
@@ -1071,8 +1292,26 @@
         <bgColor rgb="FF1F497D"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD6E4F0"/>
+        <bgColor rgb="FFD6E4F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEEF3F8"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -1110,12 +1349,67 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1165,99 +1459,199 @@
     <xf numFmtId="0" fontId="5" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="19" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="19" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="19" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="19" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="19" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="19" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="21" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="21" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="22" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="24" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="25" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="26" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="27" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="23" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="28" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="28" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="19" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="19" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="19" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="14" fillId="20" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="19" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="14" fillId="19" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="29" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="29" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="29" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="15" fillId="29" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="24" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="31" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="18" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="19" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="19" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="22" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="23" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="24" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="25" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="21" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="26" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="26" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="31" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="31" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="31" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="14" fillId="31" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Hyperlink 2" xfId="2" xr:uid="{8B207788-D8C1-4F80-8E81-707DCAD388C3}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFEEF3F8"/>
       <color rgb="FFF12F0F"/>
     </mruColors>
   </colors>
@@ -1557,7 +1951,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.33203125" style="3" customWidth="1"/>
@@ -1582,21 +1976,21 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="22" customFormat="1" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="20" t="s">
+    <row r="2" spans="1:4" s="20" customFormat="1" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="18" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="19" t="s">
         <v>5</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>7</v>
       </c>
@@ -1610,7 +2004,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -1622,7 +2016,7 @@
       </c>
       <c r="D4" s="10"/>
     </row>
-    <row r="5" spans="1:4" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
@@ -1634,7 +2028,7 @@
       </c>
       <c r="D5" s="10"/>
     </row>
-    <row r="6" spans="1:4" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>7</v>
       </c>
@@ -1648,7 +2042,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>10</v>
       </c>
@@ -1660,7 +2054,7 @@
       </c>
       <c r="D7" s="10"/>
     </row>
-    <row r="8" spans="1:4" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>10</v>
       </c>
@@ -1672,7 +2066,7 @@
       </c>
       <c r="D8" s="10"/>
     </row>
-    <row r="9" spans="1:4" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>7</v>
       </c>
@@ -1686,7 +2080,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
@@ -1698,7 +2092,7 @@
       </c>
       <c r="D10" s="10"/>
     </row>
-    <row r="11" spans="1:4" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>10</v>
       </c>
@@ -1709,6 +2103,68 @@
         <v>27</v>
       </c>
       <c r="D11" s="10"/>
+    </row>
+    <row r="12" spans="1:4" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>258</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>259</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>261</v>
+      </c>
+      <c r="D13" s="10"/>
+    </row>
+    <row r="14" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>260</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>262</v>
+      </c>
+      <c r="D14" s="10"/>
+    </row>
+    <row r="15" spans="1:4" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>263</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>265</v>
+      </c>
+      <c r="D15" s="10"/>
+    </row>
+    <row r="16" spans="1:4" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>264</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>266</v>
+      </c>
+      <c r="D16" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1718,7 +2174,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1750,7 +2206,7 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="111" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="21" t="s">
         <v>185</v>
       </c>
       <c r="B2" s="12" t="s">
@@ -1786,7 +2242,7 @@
         <v>1</v>
       </c>
       <c r="F3" s="16" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="3.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1798,7 +2254,7 @@
       <c r="F4" s="14"/>
     </row>
     <row r="5" spans="1:6" ht="69.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="23" t="s">
+      <c r="A5" s="21" t="s">
         <v>187</v>
       </c>
       <c r="B5" s="12" t="s">
@@ -1813,8 +2269,8 @@
       <c r="E5" s="12">
         <v>3</v>
       </c>
-      <c r="F5" s="23" t="s">
-        <v>219</v>
+      <c r="F5" s="21" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="58.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -1834,7 +2290,7 @@
         <v>3</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="3.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1866,7 +2322,7 @@
       </c>
     </row>
     <row r="9" spans="1:6" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="23" t="s">
+      <c r="A9" s="21" t="s">
         <v>190</v>
       </c>
       <c r="B9" s="12" t="s">
@@ -1881,8 +2337,36 @@
       <c r="E9" s="12">
         <v>3</v>
       </c>
-      <c r="F9" s="23" t="s">
+      <c r="F9" s="21" t="s">
         <v>170</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="3" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="14"/>
+      <c r="B10" s="14"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
+    </row>
+    <row r="11" spans="1:6" ht="58.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="16" t="s">
+        <v>267</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>268</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>269</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="E11" s="13">
+        <v>4</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>270</v>
       </c>
     </row>
   </sheetData>
@@ -1892,16 +2376,16 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" style="3" customWidth="1"/>
     <col min="2" max="2" width="20" style="3" customWidth="1"/>
-    <col min="3" max="3" width="22" style="3" customWidth="1"/>
+    <col min="3" max="3" width="26.77734375" style="3" customWidth="1"/>
     <col min="4" max="4" width="32" style="3" customWidth="1"/>
     <col min="5" max="5" width="38" style="3" customWidth="1"/>
     <col min="6" max="6" width="26" style="3" customWidth="1"/>
-    <col min="7" max="7" width="36" style="3" customWidth="1"/>
+    <col min="7" max="7" width="38.44140625" style="3" customWidth="1"/>
     <col min="8" max="8" width="22" style="3" customWidth="1"/>
     <col min="9" max="9" width="14" style="3" customWidth="1"/>
     <col min="10" max="10" width="22" style="3" customWidth="1"/>
@@ -1973,7 +2457,7 @@
       <c r="H2" s="13" t="s">
         <v>143</v>
       </c>
-      <c r="I2" s="19" t="s">
+      <c r="I2" s="17" t="s">
         <v>144</v>
       </c>
       <c r="J2" s="13"/>
@@ -2007,7 +2491,7 @@
       <c r="H3" s="16" t="s">
         <v>174</v>
       </c>
-      <c r="I3" s="19" t="s">
+      <c r="I3" s="17" t="s">
         <v>144</v>
       </c>
       <c r="J3" s="13"/>
@@ -2041,7 +2525,7 @@
       <c r="H4" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="I4" s="25" t="s">
+      <c r="I4" s="23" t="s">
         <v>144</v>
       </c>
       <c r="J4" s="12"/>
@@ -2057,7 +2541,7 @@
       <c r="B5" s="13" t="s">
         <v>185</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="16" t="s">
         <v>60</v>
       </c>
       <c r="D5" s="13" t="s">
@@ -2075,7 +2559,7 @@
       <c r="H5" s="13" t="s">
         <v>146</v>
       </c>
-      <c r="I5" s="19" t="s">
+      <c r="I5" s="17" t="s">
         <v>144</v>
       </c>
       <c r="J5" s="13"/>
@@ -2109,13 +2593,13 @@
       <c r="H6" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="I6" s="24" t="s">
+      <c r="I6" s="22" t="s">
         <v>148</v>
       </c>
       <c r="J6" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="K6" s="24" t="s">
+      <c r="K6" s="22" t="s">
         <v>148</v>
       </c>
       <c r="L6" s="12" t="s">
@@ -2147,7 +2631,7 @@
       <c r="H7" s="13" t="s">
         <v>150</v>
       </c>
-      <c r="I7" s="19" t="s">
+      <c r="I7" s="17" t="s">
         <v>144</v>
       </c>
       <c r="J7" s="13"/>
@@ -2181,7 +2665,7 @@
       <c r="H8" s="12" t="s">
         <v>151</v>
       </c>
-      <c r="I8" s="25" t="s">
+      <c r="I8" s="23" t="s">
         <v>144</v>
       </c>
       <c r="J8" s="12"/>
@@ -2215,7 +2699,7 @@
       <c r="H9" s="13" t="s">
         <v>151</v>
       </c>
-      <c r="I9" s="19" t="s">
+      <c r="I9" s="17" t="s">
         <v>144</v>
       </c>
       <c r="J9" s="13"/>
@@ -2225,24 +2709,24 @@
       </c>
     </row>
     <row r="10" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="62" t="s">
         <v>199</v>
       </c>
-      <c r="B10" s="18"/>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
-      <c r="G10" s="18"/>
-      <c r="H10" s="18"/>
-      <c r="I10" s="18"/>
-      <c r="J10" s="18"/>
-      <c r="K10" s="18"/>
-      <c r="L10" s="18"/>
+      <c r="B10" s="63"/>
+      <c r="C10" s="63"/>
+      <c r="D10" s="63"/>
+      <c r="E10" s="63"/>
+      <c r="F10" s="63"/>
+      <c r="G10" s="63"/>
+      <c r="H10" s="63"/>
+      <c r="I10" s="63"/>
+      <c r="J10" s="63"/>
+      <c r="K10" s="63"/>
+      <c r="L10" s="63"/>
     </row>
     <row r="11" spans="1:12" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="16" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B11" s="13" t="s">
         <v>186</v>
@@ -2265,7 +2749,7 @@
       <c r="H11" s="13" t="s">
         <v>152</v>
       </c>
-      <c r="I11" s="19" t="s">
+      <c r="I11" s="17" t="s">
         <v>144</v>
       </c>
       <c r="J11" s="13"/>
@@ -2275,20 +2759,20 @@
       </c>
     </row>
     <row r="12" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="17" t="s">
+      <c r="A12" s="62" t="s">
         <v>202</v>
       </c>
-      <c r="B12" s="18"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
-      <c r="G12" s="18"/>
-      <c r="H12" s="18"/>
-      <c r="I12" s="18"/>
-      <c r="J12" s="18"/>
-      <c r="K12" s="18"/>
-      <c r="L12" s="18"/>
+      <c r="B12" s="63"/>
+      <c r="C12" s="63"/>
+      <c r="D12" s="63"/>
+      <c r="E12" s="63"/>
+      <c r="F12" s="63"/>
+      <c r="G12" s="63"/>
+      <c r="H12" s="63"/>
+      <c r="I12" s="63"/>
+      <c r="J12" s="63"/>
+      <c r="K12" s="63"/>
+      <c r="L12" s="63"/>
     </row>
     <row r="13" spans="1:12" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="16" t="s">
@@ -2315,7 +2799,7 @@
       <c r="H13" s="13" t="s">
         <v>95</v>
       </c>
-      <c r="I13" s="19" t="s">
+      <c r="I13" s="17" t="s">
         <v>144</v>
       </c>
       <c r="J13" s="13"/>
@@ -2325,7 +2809,7 @@
       </c>
     </row>
     <row r="14" spans="1:12" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="23" t="s">
+      <c r="A14" s="21" t="s">
         <v>201</v>
       </c>
       <c r="B14" s="12" t="s">
@@ -2349,7 +2833,7 @@
       <c r="H14" s="12" t="s">
         <v>157</v>
       </c>
-      <c r="I14" s="25" t="s">
+      <c r="I14" s="23" t="s">
         <v>144</v>
       </c>
       <c r="J14" s="12"/>
@@ -2359,7 +2843,7 @@
       </c>
     </row>
     <row r="15" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="23" t="s">
+      <c r="A15" s="21" t="s">
         <v>203</v>
       </c>
       <c r="B15" s="12" t="s">
@@ -2383,7 +2867,7 @@
       <c r="H15" s="12" t="s">
         <v>158</v>
       </c>
-      <c r="I15" s="25" t="s">
+      <c r="I15" s="23" t="s">
         <v>144</v>
       </c>
       <c r="J15" s="12"/>
@@ -2393,21 +2877,21 @@
       </c>
     </row>
     <row r="16" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="17"/>
-      <c r="B16" s="18"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="18"/>
-      <c r="G16" s="18"/>
-      <c r="H16" s="18"/>
-      <c r="I16" s="18"/>
-      <c r="J16" s="18"/>
-      <c r="K16" s="18"/>
-      <c r="L16" s="18"/>
+      <c r="A16" s="62"/>
+      <c r="B16" s="63"/>
+      <c r="C16" s="63"/>
+      <c r="D16" s="63"/>
+      <c r="E16" s="63"/>
+      <c r="F16" s="63"/>
+      <c r="G16" s="63"/>
+      <c r="H16" s="63"/>
+      <c r="I16" s="63"/>
+      <c r="J16" s="63"/>
+      <c r="K16" s="63"/>
+      <c r="L16" s="63"/>
     </row>
     <row r="17" spans="1:12" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="23" t="s">
+      <c r="A17" s="21" t="s">
         <v>204</v>
       </c>
       <c r="B17" s="12" t="s">
@@ -2431,7 +2915,7 @@
       <c r="H17" s="12" t="s">
         <v>159</v>
       </c>
-      <c r="I17" s="25" t="s">
+      <c r="I17" s="23" t="s">
         <v>144</v>
       </c>
       <c r="J17" s="12"/>
@@ -2465,7 +2949,7 @@
       <c r="H18" s="13" t="s">
         <v>160</v>
       </c>
-      <c r="I18" s="19" t="s">
+      <c r="I18" s="17" t="s">
         <v>144</v>
       </c>
       <c r="J18" s="13"/>
@@ -2475,7 +2959,7 @@
       </c>
     </row>
     <row r="19" spans="1:12" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="23" t="s">
+      <c r="A19" s="21" t="s">
         <v>206</v>
       </c>
       <c r="B19" s="12" t="s">
@@ -2499,13 +2983,13 @@
       <c r="H19" s="12" t="s">
         <v>161</v>
       </c>
-      <c r="I19" s="24" t="s">
+      <c r="I19" s="22" t="s">
         <v>148</v>
       </c>
       <c r="J19" s="12" t="s">
         <v>163</v>
       </c>
-      <c r="K19" s="24" t="s">
+      <c r="K19" s="22" t="s">
         <v>148</v>
       </c>
       <c r="L19" s="12" t="s">
@@ -2513,24 +2997,24 @@
       </c>
     </row>
     <row r="20" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="17"/>
-      <c r="B20" s="18"/>
-      <c r="C20" s="18"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="18"/>
-      <c r="F20" s="18"/>
-      <c r="G20" s="18"/>
-      <c r="H20" s="18"/>
-      <c r="I20" s="18"/>
-      <c r="J20" s="18"/>
-      <c r="K20" s="18"/>
-      <c r="L20" s="18"/>
+      <c r="A20" s="62"/>
+      <c r="B20" s="63"/>
+      <c r="C20" s="63"/>
+      <c r="D20" s="63"/>
+      <c r="E20" s="63"/>
+      <c r="F20" s="63"/>
+      <c r="G20" s="63"/>
+      <c r="H20" s="63"/>
+      <c r="I20" s="63"/>
+      <c r="J20" s="63"/>
+      <c r="K20" s="63"/>
+      <c r="L20" s="63"/>
     </row>
     <row r="21" spans="1:12" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="23" t="s">
+      <c r="A21" s="21" t="s">
         <v>207</v>
       </c>
-      <c r="B21" s="23" t="s">
+      <c r="B21" s="21" t="s">
         <v>189</v>
       </c>
       <c r="C21" s="12" t="s">
@@ -2551,7 +3035,7 @@
       <c r="H21" s="12" t="s">
         <v>164</v>
       </c>
-      <c r="I21" s="25" t="s">
+      <c r="I21" s="23" t="s">
         <v>144</v>
       </c>
       <c r="J21" s="12"/>
@@ -2585,7 +3069,7 @@
       <c r="H22" s="13" t="s">
         <v>165</v>
       </c>
-      <c r="I22" s="19" t="s">
+      <c r="I22" s="17" t="s">
         <v>144</v>
       </c>
       <c r="J22" s="13"/>
@@ -2595,10 +3079,10 @@
       </c>
     </row>
     <row r="23" spans="1:12" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="23" t="s">
+      <c r="A23" s="21" t="s">
         <v>209</v>
       </c>
-      <c r="B23" s="23" t="s">
+      <c r="B23" s="21" t="s">
         <v>189</v>
       </c>
       <c r="C23" s="12" t="s">
@@ -2619,7 +3103,7 @@
       <c r="H23" s="12" t="s">
         <v>166</v>
       </c>
-      <c r="I23" s="25" t="s">
+      <c r="I23" s="23" t="s">
         <v>144</v>
       </c>
       <c r="J23" s="12"/>
@@ -2629,20 +3113,20 @@
       </c>
     </row>
     <row r="24" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="17" t="s">
+      <c r="A24" s="62" t="s">
         <v>212</v>
       </c>
-      <c r="B24" s="18"/>
-      <c r="C24" s="18"/>
-      <c r="D24" s="18"/>
-      <c r="E24" s="18"/>
-      <c r="F24" s="18"/>
-      <c r="G24" s="18"/>
-      <c r="H24" s="18"/>
-      <c r="I24" s="18"/>
-      <c r="J24" s="18"/>
-      <c r="K24" s="18"/>
-      <c r="L24" s="18"/>
+      <c r="B24" s="63"/>
+      <c r="C24" s="63"/>
+      <c r="D24" s="63"/>
+      <c r="E24" s="63"/>
+      <c r="F24" s="63"/>
+      <c r="G24" s="63"/>
+      <c r="H24" s="63"/>
+      <c r="I24" s="63"/>
+      <c r="J24" s="63"/>
+      <c r="K24" s="63"/>
+      <c r="L24" s="63"/>
     </row>
     <row r="25" spans="1:12" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="16" t="s">
@@ -2669,7 +3153,7 @@
       <c r="H25" s="16" t="s">
         <v>168</v>
       </c>
-      <c r="I25" s="26" t="s">
+      <c r="I25" s="24" t="s">
         <v>144</v>
       </c>
       <c r="J25" s="13"/>
@@ -2679,10 +3163,10 @@
       </c>
     </row>
     <row r="26" spans="1:12" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="23" t="s">
+      <c r="A26" s="21" t="s">
         <v>211</v>
       </c>
-      <c r="B26" s="23" t="s">
+      <c r="B26" s="21" t="s">
         <v>190</v>
       </c>
       <c r="C26" s="12" t="s">
@@ -2700,10 +3184,10 @@
       <c r="G26" s="12" t="s">
         <v>137</v>
       </c>
-      <c r="H26" s="23" t="s">
+      <c r="H26" s="21" t="s">
         <v>164</v>
       </c>
-      <c r="I26" s="27" t="s">
+      <c r="I26" s="25" t="s">
         <v>144</v>
       </c>
       <c r="J26" s="12"/>
@@ -2737,7 +3221,7 @@
       <c r="H27" s="16" t="s">
         <v>169</v>
       </c>
-      <c r="I27" s="26" t="s">
+      <c r="I27" s="24" t="s">
         <v>144</v>
       </c>
       <c r="J27" s="13"/>
@@ -2746,8 +3230,161 @@
         <v>47</v>
       </c>
     </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A28" s="62" t="s">
+        <v>212</v>
+      </c>
+      <c r="B28" s="63"/>
+      <c r="C28" s="63"/>
+      <c r="D28" s="63"/>
+      <c r="E28" s="63"/>
+      <c r="F28" s="63"/>
+      <c r="G28" s="63"/>
+      <c r="H28" s="63"/>
+      <c r="I28" s="63"/>
+      <c r="J28" s="63"/>
+      <c r="K28" s="63"/>
+      <c r="L28" s="63"/>
+    </row>
+    <row r="29" spans="1:12" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A29" s="16" t="s">
+        <v>271</v>
+      </c>
+      <c r="B29" s="16" t="s">
+        <v>267</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>275</v>
+      </c>
+      <c r="D29" s="13" t="s">
+        <v>276</v>
+      </c>
+      <c r="E29" s="13" t="s">
+        <v>277</v>
+      </c>
+      <c r="F29" s="13" t="s">
+        <v>279</v>
+      </c>
+      <c r="G29" s="13" t="s">
+        <v>278</v>
+      </c>
+      <c r="H29" s="16" t="s">
+        <v>280</v>
+      </c>
+      <c r="I29" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="J29" s="13"/>
+      <c r="K29" s="13"/>
+      <c r="L29" s="13" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A30" s="21" t="s">
+        <v>272</v>
+      </c>
+      <c r="B30" s="21" t="s">
+        <v>267</v>
+      </c>
+      <c r="C30" s="12" t="s">
+        <v>275</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>282</v>
+      </c>
+      <c r="E30" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="F30" s="12" t="s">
+        <v>284</v>
+      </c>
+      <c r="G30" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="H30" s="21" t="s">
+        <v>286</v>
+      </c>
+      <c r="I30" s="25" t="s">
+        <v>144</v>
+      </c>
+      <c r="J30" s="12"/>
+      <c r="K30" s="12"/>
+      <c r="L30" s="12" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A31" s="16" t="s">
+        <v>273</v>
+      </c>
+      <c r="B31" s="16" t="s">
+        <v>267</v>
+      </c>
+      <c r="C31" s="13" t="s">
+        <v>275</v>
+      </c>
+      <c r="D31" s="13" t="s">
+        <v>287</v>
+      </c>
+      <c r="E31" s="13" t="s">
+        <v>289</v>
+      </c>
+      <c r="F31" s="13" t="s">
+        <v>290</v>
+      </c>
+      <c r="G31" s="13" t="s">
+        <v>288</v>
+      </c>
+      <c r="H31" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="I31" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="J31" s="13"/>
+      <c r="K31" s="13"/>
+      <c r="L31" s="13" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A32" s="16" t="s">
+        <v>274</v>
+      </c>
+      <c r="B32" s="16" t="s">
+        <v>267</v>
+      </c>
+      <c r="C32" s="13" t="s">
+        <v>275</v>
+      </c>
+      <c r="D32" s="13" t="s">
+        <v>292</v>
+      </c>
+      <c r="E32" s="13" t="s">
+        <v>294</v>
+      </c>
+      <c r="F32" s="13" t="s">
+        <v>293</v>
+      </c>
+      <c r="G32" s="13" t="s">
+        <v>295</v>
+      </c>
+      <c r="H32" s="16" t="s">
+        <v>296</v>
+      </c>
+      <c r="I32" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="J32" s="13"/>
+      <c r="K32" s="13"/>
+      <c r="L32" s="13" t="s">
+        <v>299</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
+    <mergeCell ref="A28:L28"/>
     <mergeCell ref="A24:L24"/>
     <mergeCell ref="A12:L12"/>
     <mergeCell ref="A10:L10"/>
@@ -2791,43 +3428,43 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="49.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="26" t="s">
         <v>214</v>
       </c>
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="27" t="s">
         <v>181</v>
       </c>
-      <c r="C2" s="29" t="s">
+      <c r="C2" s="27" t="s">
         <v>182</v>
       </c>
-      <c r="D2" s="30" t="s">
+      <c r="D2" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="32" t="s">
+      <c r="E2" s="30" t="s">
+        <v>220</v>
+      </c>
+      <c r="F2" s="29" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="26" t="s">
+        <v>215</v>
+      </c>
+      <c r="B3" s="27" t="s">
+        <v>183</v>
+      </c>
+      <c r="C3" s="27" t="s">
+        <v>184</v>
+      </c>
+      <c r="D3" s="28" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="30" t="s">
         <v>221</v>
       </c>
-      <c r="F2" s="31" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="51" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="28" t="s">
-        <v>215</v>
-      </c>
-      <c r="B3" s="29" t="s">
-        <v>183</v>
-      </c>
-      <c r="C3" s="29" t="s">
-        <v>184</v>
-      </c>
-      <c r="D3" s="30" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" s="32" t="s">
-        <v>222</v>
-      </c>
-      <c r="F3" s="31" t="s">
-        <v>244</v>
+      <c r="F3" s="29" t="s">
+        <v>243</v>
       </c>
     </row>
   </sheetData>
@@ -2841,7 +3478,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2964BC42-3F95-4102-8105-8383C1296CE9}">
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -2854,30 +3491,30 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="44" t="s">
+        <v>222</v>
+      </c>
+      <c r="B1" s="44" t="s">
         <v>223</v>
       </c>
-      <c r="B1" s="44" t="s">
+      <c r="C1" s="44" t="s">
         <v>224</v>
       </c>
-      <c r="C1" s="44" t="s">
+      <c r="D1" s="44" t="s">
         <v>225</v>
       </c>
-      <c r="D1" s="44" t="s">
+      <c r="E1" s="44" t="s">
         <v>226</v>
       </c>
-      <c r="E1" s="44" t="s">
+      <c r="F1" s="44" t="s">
         <v>227</v>
-      </c>
-      <c r="F1" s="44" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="33" t="s">
+        <v>231</v>
+      </c>
+      <c r="B2" s="33" t="s">
         <v>232</v>
-      </c>
-      <c r="B2" s="33" t="s">
-        <v>233</v>
       </c>
       <c r="C2" s="33" t="s">
         <v>185</v>
@@ -2886,10 +3523,10 @@
         <v>191</v>
       </c>
       <c r="E2" s="38" t="s">
+        <v>228</v>
+      </c>
+      <c r="F2" s="35" t="s">
         <v>229</v>
-      </c>
-      <c r="F2" s="35" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -2900,10 +3537,10 @@
         <v>192</v>
       </c>
       <c r="E3" s="39" t="s">
+        <v>228</v>
+      </c>
+      <c r="F3" s="36" t="s">
         <v>229</v>
-      </c>
-      <c r="F3" s="36" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -2914,10 +3551,10 @@
         <v>193</v>
       </c>
       <c r="E4" s="39" t="s">
+        <v>228</v>
+      </c>
+      <c r="F4" s="36" t="s">
         <v>229</v>
-      </c>
-      <c r="F4" s="36" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
@@ -2928,10 +3565,10 @@
         <v>194</v>
       </c>
       <c r="E5" s="38" t="s">
+        <v>228</v>
+      </c>
+      <c r="F5" s="35" t="s">
         <v>229</v>
-      </c>
-      <c r="F5" s="35" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
@@ -2942,7 +3579,7 @@
         <v>195</v>
       </c>
       <c r="E6" s="40" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F6" s="37" t="s">
         <v>214</v>
@@ -2956,10 +3593,10 @@
         <v>196</v>
       </c>
       <c r="E7" s="38" t="s">
+        <v>228</v>
+      </c>
+      <c r="F7" s="35" t="s">
         <v>229</v>
-      </c>
-      <c r="F7" s="35" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -2970,10 +3607,10 @@
         <v>197</v>
       </c>
       <c r="E8" s="39" t="s">
+        <v>228</v>
+      </c>
+      <c r="F8" s="36" t="s">
         <v>229</v>
-      </c>
-      <c r="F8" s="36" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -2984,38 +3621,38 @@
         <v>198</v>
       </c>
       <c r="E9" s="38" t="s">
+        <v>228</v>
+      </c>
+      <c r="F9" s="35" t="s">
         <v>229</v>
-      </c>
-      <c r="F9" s="35" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="34" t="s">
+        <v>233</v>
+      </c>
+      <c r="B10" s="34" t="s">
         <v>234</v>
-      </c>
-      <c r="B10" s="34" t="s">
-        <v>235</v>
       </c>
       <c r="C10" s="34" t="s">
         <v>186</v>
       </c>
       <c r="D10" s="34" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="E10" s="39" t="s">
+        <v>228</v>
+      </c>
+      <c r="F10" s="36" t="s">
         <v>229</v>
-      </c>
-      <c r="F10" s="36" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="34" t="s">
+        <v>235</v>
+      </c>
+      <c r="B11" s="34" t="s">
         <v>236</v>
-      </c>
-      <c r="B11" s="34" t="s">
-        <v>237</v>
       </c>
       <c r="C11" s="34" t="s">
         <v>187</v>
@@ -3024,10 +3661,10 @@
         <v>200</v>
       </c>
       <c r="E11" s="39" t="s">
+        <v>228</v>
+      </c>
+      <c r="F11" s="36" t="s">
         <v>229</v>
-      </c>
-      <c r="F11" s="36" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
@@ -3038,10 +3675,10 @@
         <v>201</v>
       </c>
       <c r="E12" s="38" t="s">
+        <v>228</v>
+      </c>
+      <c r="F12" s="35" t="s">
         <v>229</v>
-      </c>
-      <c r="F12" s="35" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -3052,18 +3689,18 @@
         <v>203</v>
       </c>
       <c r="E13" s="39" t="s">
+        <v>228</v>
+      </c>
+      <c r="F13" s="36" t="s">
         <v>229</v>
-      </c>
-      <c r="F13" s="36" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="33" t="s">
+        <v>237</v>
+      </c>
+      <c r="B14" s="33" t="s">
         <v>238</v>
-      </c>
-      <c r="B14" s="33" t="s">
-        <v>239</v>
       </c>
       <c r="C14" s="33" t="s">
         <v>188</v>
@@ -3072,10 +3709,10 @@
         <v>204</v>
       </c>
       <c r="E14" s="38" t="s">
+        <v>228</v>
+      </c>
+      <c r="F14" s="35" t="s">
         <v>229</v>
-      </c>
-      <c r="F14" s="35" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -3086,10 +3723,10 @@
         <v>205</v>
       </c>
       <c r="E15" s="39" t="s">
+        <v>228</v>
+      </c>
+      <c r="F15" s="36" t="s">
         <v>229</v>
-      </c>
-      <c r="F15" s="36" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -3100,18 +3737,18 @@
         <v>206</v>
       </c>
       <c r="E16" s="41" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F16" s="42" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="34" t="s">
+        <v>239</v>
+      </c>
+      <c r="B17" s="34" t="s">
         <v>240</v>
-      </c>
-      <c r="B17" s="34" t="s">
-        <v>241</v>
       </c>
       <c r="C17" s="34" t="s">
         <v>189</v>
@@ -3120,10 +3757,10 @@
         <v>207</v>
       </c>
       <c r="E17" s="39" t="s">
+        <v>228</v>
+      </c>
+      <c r="F17" s="36" t="s">
         <v>229</v>
-      </c>
-      <c r="F17" s="36" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -3134,10 +3771,10 @@
         <v>208</v>
       </c>
       <c r="E18" s="38" t="s">
+        <v>228</v>
+      </c>
+      <c r="F18" s="35" t="s">
         <v>229</v>
-      </c>
-      <c r="F18" s="35" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -3148,18 +3785,18 @@
         <v>209</v>
       </c>
       <c r="E19" s="39" t="s">
+        <v>228</v>
+      </c>
+      <c r="F19" s="36" t="s">
         <v>229</v>
-      </c>
-      <c r="F19" s="36" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="33" t="s">
+        <v>241</v>
+      </c>
+      <c r="B20" s="33" t="s">
         <v>242</v>
-      </c>
-      <c r="B20" s="33" t="s">
-        <v>243</v>
       </c>
       <c r="C20" s="33" t="s">
         <v>190</v>
@@ -3168,10 +3805,10 @@
         <v>210</v>
       </c>
       <c r="E20" s="38" t="s">
+        <v>228</v>
+      </c>
+      <c r="F20" s="35" t="s">
         <v>229</v>
-      </c>
-      <c r="F20" s="35" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
@@ -3182,27 +3819,395 @@
         <v>211</v>
       </c>
       <c r="E21" s="39" t="s">
+        <v>228</v>
+      </c>
+      <c r="F21" s="36" t="s">
         <v>229</v>
       </c>
-      <c r="F21" s="36" t="s">
-        <v>230</v>
-      </c>
     </row>
     <row r="22" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="33"/>
-      <c r="B22" s="33"/>
-      <c r="C22" s="33"/>
-      <c r="D22" s="33" t="s">
+      <c r="A22" s="69"/>
+      <c r="B22" s="69"/>
+      <c r="C22" s="69"/>
+      <c r="D22" s="69" t="s">
         <v>213</v>
       </c>
-      <c r="E22" s="38" t="s">
+      <c r="E22" s="68" t="s">
+        <v>228</v>
+      </c>
+      <c r="F22" s="70" t="s">
         <v>229</v>
       </c>
-      <c r="F22" s="35" t="s">
-        <v>230</v>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" s="73" t="s">
+        <v>300</v>
+      </c>
+      <c r="B23" s="71" t="s">
+        <v>301</v>
+      </c>
+      <c r="C23" s="71" t="s">
+        <v>267</v>
+      </c>
+      <c r="D23" s="71" t="s">
+        <v>271</v>
+      </c>
+      <c r="E23" s="72" t="s">
+        <v>228</v>
+      </c>
+      <c r="F23" s="71" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="71"/>
+      <c r="B24" s="71"/>
+      <c r="C24" s="71"/>
+      <c r="D24" s="71" t="s">
+        <v>272</v>
+      </c>
+      <c r="E24" s="72" t="s">
+        <v>228</v>
+      </c>
+      <c r="F24" s="71" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" s="71"/>
+      <c r="B25" s="71"/>
+      <c r="C25" s="71"/>
+      <c r="D25" s="71" t="s">
+        <v>273</v>
+      </c>
+      <c r="E25" s="72" t="s">
+        <v>228</v>
+      </c>
+      <c r="F25" s="71" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" s="71"/>
+      <c r="B26" s="71"/>
+      <c r="C26" s="71"/>
+      <c r="D26" s="71" t="s">
+        <v>274</v>
+      </c>
+      <c r="E26" s="72" t="s">
+        <v>228</v>
+      </c>
+      <c r="F26" s="71" t="s">
+        <v>229</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB572326-E878-4020-9542-81828AEF480C}">
+  <dimension ref="A1:I10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="18.109375" customWidth="1"/>
+    <col min="2" max="2" width="29.21875" customWidth="1"/>
+    <col min="3" max="3" width="11.6640625" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" customWidth="1"/>
+    <col min="5" max="5" width="10.88671875" customWidth="1"/>
+    <col min="6" max="6" width="12.88671875" customWidth="1"/>
+    <col min="7" max="7" width="14.21875" customWidth="1"/>
+    <col min="8" max="8" width="14.33203125" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="64" t="s">
+        <v>244</v>
+      </c>
+      <c r="B1" s="65"/>
+      <c r="C1" s="65"/>
+      <c r="D1" s="65"/>
+      <c r="E1" s="65"/>
+      <c r="F1" s="65"/>
+      <c r="G1" s="65"/>
+      <c r="H1" s="65"/>
+      <c r="I1" s="65"/>
+    </row>
+    <row r="2" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="48" t="s">
+        <v>245</v>
+      </c>
+      <c r="B2" s="48" t="s">
+        <v>246</v>
+      </c>
+      <c r="C2" s="48" t="s">
+        <v>247</v>
+      </c>
+      <c r="D2" s="48" t="s">
+        <v>248</v>
+      </c>
+      <c r="E2" s="48" t="s">
+        <v>249</v>
+      </c>
+      <c r="F2" s="48" t="s">
+        <v>250</v>
+      </c>
+      <c r="G2" s="48" t="s">
+        <v>251</v>
+      </c>
+      <c r="H2" s="48" t="s">
+        <v>252</v>
+      </c>
+      <c r="I2" s="48" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="49" t="s">
+        <v>253</v>
+      </c>
+      <c r="B3" s="50" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" s="51">
+        <v>8</v>
+      </c>
+      <c r="D3" s="52">
+        <v>7</v>
+      </c>
+      <c r="E3" s="53">
+        <v>1</v>
+      </c>
+      <c r="F3" s="51">
+        <v>8</v>
+      </c>
+      <c r="G3" s="54">
+        <f t="shared" ref="G3:G10" si="0">IF(C3=0,0,D3/C3)</f>
+        <v>0.875</v>
+      </c>
+      <c r="H3" s="54">
+        <f t="shared" ref="H3:H10" si="1">IF(C3=0,0,E3/C3)</f>
+        <v>0.125</v>
+      </c>
+      <c r="I3" s="54">
+        <f t="shared" ref="I3:I10" si="2">IF(C3=0,0,F3/C3)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="46"/>
+      <c r="B4" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" s="45" t="s">
+        <v>302</v>
+      </c>
+      <c r="D4" s="55">
+        <v>1</v>
+      </c>
+      <c r="E4" s="47">
+        <v>0</v>
+      </c>
+      <c r="F4" s="45">
+        <v>1</v>
+      </c>
+      <c r="G4" s="56">
+        <v>1</v>
+      </c>
+      <c r="H4" s="56">
+        <v>0</v>
+      </c>
+      <c r="I4" s="56">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="50"/>
+      <c r="B5" s="50" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" s="51">
+        <v>3</v>
+      </c>
+      <c r="D5" s="52">
+        <v>3</v>
+      </c>
+      <c r="E5" s="32">
+        <v>0</v>
+      </c>
+      <c r="F5" s="51">
+        <v>3</v>
+      </c>
+      <c r="G5" s="54">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="H5" s="54">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I5" s="54">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="46"/>
+      <c r="B6" s="46" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6" s="45">
+        <v>3</v>
+      </c>
+      <c r="D6" s="55">
+        <v>2</v>
+      </c>
+      <c r="E6" s="47">
+        <v>1</v>
+      </c>
+      <c r="F6" s="45">
+        <v>3</v>
+      </c>
+      <c r="G6" s="56">
+        <f t="shared" si="0"/>
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="H6" s="56">
+        <f t="shared" si="1"/>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="I6" s="56">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="50"/>
+      <c r="B7" s="50" t="s">
+        <v>256</v>
+      </c>
+      <c r="C7" s="51">
+        <v>3</v>
+      </c>
+      <c r="D7" s="52">
+        <v>3</v>
+      </c>
+      <c r="E7" s="32">
+        <v>0</v>
+      </c>
+      <c r="F7" s="51">
+        <v>3</v>
+      </c>
+      <c r="G7" s="54">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="H7" s="54">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I7" s="54">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" s="61" customFormat="1" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="46"/>
+      <c r="B8" s="46" t="s">
+        <v>254</v>
+      </c>
+      <c r="C8" s="45">
+        <v>3</v>
+      </c>
+      <c r="D8" s="55">
+        <v>3</v>
+      </c>
+      <c r="E8" s="31">
+        <v>0</v>
+      </c>
+      <c r="F8" s="45">
+        <v>3</v>
+      </c>
+      <c r="G8" s="56">
+        <f t="shared" ref="G8" si="3">IF(C8=0,0,D8/C8)</f>
+        <v>1</v>
+      </c>
+      <c r="H8" s="56">
+        <f t="shared" ref="H8" si="4">IF(C8=0,0,E8/C8)</f>
+        <v>0</v>
+      </c>
+      <c r="I8" s="56">
+        <f t="shared" ref="I8" si="5">IF(C8=0,0,F8/C8)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="74"/>
+      <c r="B9" s="74" t="s">
+        <v>269</v>
+      </c>
+      <c r="C9" s="75">
+        <v>4</v>
+      </c>
+      <c r="D9" s="76">
+        <v>4</v>
+      </c>
+      <c r="E9" s="77">
+        <v>0</v>
+      </c>
+      <c r="F9" s="75">
+        <v>4</v>
+      </c>
+      <c r="G9" s="78">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="H9" s="78">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I9" s="78">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A10" s="66" t="s">
+        <v>255</v>
+      </c>
+      <c r="B10" s="67"/>
+      <c r="C10" s="57">
+        <v>25</v>
+      </c>
+      <c r="D10" s="58">
+        <v>23</v>
+      </c>
+      <c r="E10" s="59">
+        <v>2</v>
+      </c>
+      <c r="F10" s="57">
+        <v>25</v>
+      </c>
+      <c r="G10" s="60">
+        <f t="shared" si="0"/>
+        <v>0.92</v>
+      </c>
+      <c r="H10" s="60">
+        <f t="shared" si="1"/>
+        <v>0.08</v>
+      </c>
+      <c r="I10" s="60">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A10:B10"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>